<commit_message>
Updated Targets for Calibration including Solano/Napa and North Bay targets
The targets were generating using the travel-diary-survey-tools (commit id: b42b819dd997daac30213374409f53f7546619e9)
</commit_message>
<xml_diff>
--- a/utilities/calibration/workbook_templates/04_CoordinatedDailyActivityPattern_2023_blank.xlsx
+++ b/utilities/calibration/workbook_templates/04_CoordinatedDailyActivityPattern_2023_blank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\travel-model-one\utilities\calibration\workbook_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{152E2EC8-5B39-4152-8450-112B8A6E21C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C1F13A-4898-48DB-90CD-1A7ABDD79E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="calibration" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId7"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -111,10 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="45">
-  <si>
-    <t>freq</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="50">
   <si>
     <t>H</t>
   </si>
@@ -242,10 +239,28 @@
     <t>activity_pattern</t>
   </si>
   <si>
-    <t>Source: M:/Development/Travel Model One/Calibration/Version 1.7/2023_BATS_Summaries/pipeline_mt_20260507/ctramp_2023/BATS_Summaries/dap_summaries.csv</t>
+    <t xml:space="preserve">**BATS 2023 was under-reporting mandatory tours for students under 18, most likely due to proxy reporting. As a result, we will not be using BATS CDAP share for students under 18 and keep the targets from the previous calibration </t>
   </si>
   <si>
-    <t xml:space="preserve">**BATS 2023 was under-reporting mandatory tours for students under 18, most likely due to proxy reporting. As a result, we will not be using BATS CDAP share for students under 18 and keep the targets from the previous calibration </t>
+    <t>num_pers</t>
+  </si>
+  <si>
+    <t>Source: M:/Development/Travel Model One/Calibration/Version 1.7/2023_BATS_Summaries/pipeline_mt_20260623_NoMon_rmo/ctramp_2023/BATS_Summaries/dap_summaries.csv</t>
+  </si>
+  <si>
+    <t>num_records</t>
+  </si>
+  <si>
+    <t>Solano/Napa</t>
+  </si>
+  <si>
+    <t>Source: M:/Development/Travel Model One/Calibration/Version 1.7/2023_BATS_Summaries/pipeline_mt_20260623_NoMon_rmo/ctramp_2023/BATS_Summaries/BATS2023_person_type_summary_solano_napa.csv</t>
+  </si>
+  <si>
+    <t>North Bay</t>
+  </si>
+  <si>
+    <t>Source: M:/Development/Travel Model One/Calibration/Version 1.7/2023_BATS_Summaries/pipeline_mt_20260623_NoMon_rmo/ctramp_2023/BATS_Summaries/BATS2023_person_type_summary_north_bay.csv</t>
   </si>
 </sst>
 </file>
@@ -600,12 +615,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{83A0AB90-23CF-41D1-8C82-7D6057588797}"/>
     <cellStyle name="Percent 2" xfId="2" xr:uid="{CB21E4C0-D945-46EE-9A00-BE0A2B1C7632}"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <sz val="10"/>
-      </font>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <sz val="10"/>
@@ -2136,7 +2146,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Melody Tsao" refreshedDate="46175.681245138891" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="22" xr:uid="{FD949337-A2E9-4B56-88F0-0CD92EE5399C}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="C2:E24" sheet="BATS 2023"/>
+    <worksheetSource ref="C2:E23" sheet="BATS 2023"/>
   </cacheSource>
   <cacheFields count="3">
     <cacheField name="person_type" numFmtId="0">
@@ -2286,7 +2296,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{425DF6BC-449A-4A16-B9F3-1C22AC562EC2}" name="PivotTable5" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{425DF6BC-449A-4A16-B9F3-1C22AC562EC2}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="I5:M15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -2365,7 +2375,7 @@
     <dataField name="Sum of freq" fld="2" baseField="0" baseItem="0" numFmtId="3"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="1">
+    <format dxfId="0">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -2668,65 +2678,65 @@
   <sheetData>
     <row r="2" spans="1:16" s="68" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B2" s="69" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H2" s="69" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M2" s="69" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="C3" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>3</v>
-      </c>
       <c r="E3" s="8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="H4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="J4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="K4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="M4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="N4" s="7" t="s">
+      <c r="O4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="P4" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
@@ -2734,7 +2744,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" s="9">
         <f>GETPIVOTDATA("freq",'BATS 2023'!$I$5,"person_type",$A5,"activity_pattern",C$3)</f>
@@ -2790,7 +2800,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" s="12">
         <f>GETPIVOTDATA("freq",'BATS 2023'!$I$5,"person_type",$A6,"activity_pattern",C$3)</f>
@@ -2846,7 +2856,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="12">
         <f>GETPIVOTDATA("freq",'BATS 2023'!$I$5,"person_type",$A7,"activity_pattern",C$3)</f>
@@ -2902,7 +2912,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="12">
         <f>GETPIVOTDATA("freq",'BATS 2023'!$I$5,"person_type",$A8,"activity_pattern",C$3)</f>
@@ -2958,7 +2968,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" s="12">
         <f>GETPIVOTDATA("freq",'BATS 2023'!$I$5,"person_type",$A9,"activity_pattern",C$3)</f>
@@ -3014,7 +3024,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" s="12">
         <f>GETPIVOTDATA("freq",'BATS 2023'!$I$5,"person_type",$A10,"activity_pattern",C$3)</f>
@@ -3070,7 +3080,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11" s="12">
         <f>GETPIVOTDATA("freq",'BATS 2023'!$I$5,"person_type",$A11,"activity_pattern",C$3)</f>
@@ -3126,7 +3136,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12" s="14">
         <f>GETPIVOTDATA("freq",'BATS 2023'!$I$5,"person_type",$A12,"activity_pattern",C$3)</f>
@@ -3179,7 +3189,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B13" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13" s="5">
         <f>GETPIVOTDATA("freq",'BATS 2023'!$I$5,"activity_pattern",C$3)</f>
@@ -3232,48 +3242,48 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="F16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="H16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="J16" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J16" s="7" t="s">
+      <c r="K16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="M16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="N16" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="N16" s="7" t="s">
+      <c r="O16" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="O16" s="7" t="s">
+      <c r="P16" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C17" s="18">
         <f>C5/$F5</f>
@@ -3326,7 +3336,7 @@
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B18" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C18" s="21">
         <f t="shared" ref="C18:F18" si="11">C6/$F6</f>
@@ -3379,7 +3389,7 @@
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C19" s="21">
         <f t="shared" ref="C19:F19" si="14">C7/$F7</f>
@@ -3432,7 +3442,7 @@
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B20" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C20" s="21">
         <f t="shared" ref="C20:F20" si="16">C8/$F8</f>
@@ -3485,7 +3495,7 @@
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B21" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C21" s="21">
         <f t="shared" ref="C21:F21" si="18">C9/$F9</f>
@@ -3538,7 +3548,7 @@
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B22" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C22" s="21">
         <f t="shared" ref="C22:F22" si="20">C10/$F10</f>
@@ -3591,7 +3601,7 @@
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C23" s="21">
         <f t="shared" ref="C23:F23" si="22">C11/$F11</f>
@@ -3644,7 +3654,7 @@
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B24" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C24" s="23">
         <f t="shared" ref="C24:F24" si="24">C12/$F12</f>
@@ -3697,7 +3707,7 @@
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C25" s="17">
         <f t="shared" ref="C25:F25" si="26">C13/$F13</f>
@@ -3750,7 +3760,7 @@
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B27" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C27" s="32">
         <v>0</v>
@@ -3758,58 +3768,58 @@
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B29" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C29" s="29"/>
       <c r="D29" s="29"/>
       <c r="E29" s="29"/>
       <c r="F29" s="28"/>
       <c r="H29" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M29" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="M29" s="6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="30" spans="2:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B30" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C30" s="44" t="s">
+      <c r="D30" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D30" s="44" t="s">
+      <c r="E30" s="44" t="s">
         <v>18</v>
-      </c>
-      <c r="E30" s="44" t="s">
-        <v>19</v>
       </c>
       <c r="F30" s="45"/>
       <c r="G30" s="7"/>
       <c r="H30" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="I30" s="44" t="s">
+      <c r="J30" s="44" t="s">
         <v>18</v>
-      </c>
-      <c r="J30" s="44" t="s">
-        <v>19</v>
       </c>
       <c r="K30" s="7"/>
       <c r="L30" s="7"/>
       <c r="M30" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="N30" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="N30" s="44" t="s">
+      <c r="O30" s="44" t="s">
         <v>18</v>
-      </c>
-      <c r="O30" s="44" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="31" spans="2:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B31" s="30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C31" s="33">
         <f>[1]OnePerson!G31</f>
@@ -3842,7 +3852,7 @@
     </row>
     <row r="32" spans="2:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B32" s="30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C32" s="36">
         <f>[1]OnePerson!G32</f>
@@ -3875,7 +3885,7 @@
     </row>
     <row r="33" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B33" s="30" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C33" s="36">
         <f>[1]OnePerson!G33</f>
@@ -3908,7 +3918,7 @@
     </row>
     <row r="34" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B34" s="30" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C34" s="36">
         <f>[1]OnePerson!G34</f>
@@ -3938,7 +3948,7 @@
     </row>
     <row r="35" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B35" s="30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C35" s="36">
         <f>[1]OnePerson!G35</f>
@@ -3968,7 +3978,7 @@
     </row>
     <row r="36" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B36" s="30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C36" s="36">
         <f>[1]OnePerson!G36</f>
@@ -4001,7 +4011,7 @@
     </row>
     <row r="37" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B37" s="30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C37" s="36">
         <f>[1]OnePerson!G37</f>
@@ -4034,7 +4044,7 @@
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B38" s="30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C38" s="38">
         <f>[1]OnePerson!G38</f>
@@ -4067,65 +4077,65 @@
     </row>
     <row r="41" spans="1:16" s="68" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B41" s="69" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H41" s="69" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M41" s="69" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="C42" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D42" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D42" s="8" t="s">
-        <v>3</v>
-      </c>
       <c r="E42" s="8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B43" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C43" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="D43" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="E43" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E43" s="7" t="s">
+      <c r="F43" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F43" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="H43" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I43" s="7" t="s">
+      <c r="J43" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J43" s="7" t="s">
+      <c r="K43" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K43" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="M43" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="N43" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="N43" s="7" t="s">
+      <c r="O43" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="O43" s="7" t="s">
+      <c r="P43" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="P43" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.2">
@@ -4133,7 +4143,7 @@
         <v>1</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C44" s="9">
         <f>'TM1 v03 Targets'!B41</f>
@@ -4189,7 +4199,7 @@
         <v>2</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C45" s="12">
         <f>'TM1 v03 Targets'!B42</f>
@@ -4245,7 +4255,7 @@
         <v>3</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C46" s="12">
         <f>'TM1 v03 Targets'!B43</f>
@@ -4301,7 +4311,7 @@
         <v>4</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C47" s="12">
         <f>'TM1 v03 Targets'!B44</f>
@@ -4357,7 +4367,7 @@
         <v>5</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C48" s="12">
         <f>'TM1 v03 Targets'!B45</f>
@@ -4413,7 +4423,7 @@
         <v>6</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C49" s="12">
         <f>'TM1 v03 Targets'!B46</f>
@@ -4469,7 +4479,7 @@
         <v>7</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C50" s="12">
         <f>'TM1 v03 Targets'!B47</f>
@@ -4525,7 +4535,7 @@
         <v>8</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C51" s="14">
         <f>'TM1 v03 Targets'!B48</f>
@@ -4578,7 +4588,7 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B52" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C52" s="5">
         <f>SUM(C44:C51)</f>
@@ -4631,48 +4641,48 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B55" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C55" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C55" s="7" t="s">
+      <c r="D55" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D55" s="7" t="s">
+      <c r="E55" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E55" s="7" t="s">
+      <c r="F55" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F55" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="H55" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I55" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I55" s="7" t="s">
+      <c r="J55" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J55" s="7" t="s">
+      <c r="K55" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K55" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="M55" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="N55" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="N55" s="7" t="s">
+      <c r="O55" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="O55" s="7" t="s">
+      <c r="P55" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="P55" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B56" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C56" s="18">
         <f>C44/$F44</f>
@@ -4725,7 +4735,7 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B57" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C57" s="21">
         <f t="shared" ref="C57:F57" si="42">C45/$F45</f>
@@ -4778,7 +4788,7 @@
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B58" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C58" s="21">
         <f t="shared" ref="C58:F58" si="45">C46/$F46</f>
@@ -4831,7 +4841,7 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B59" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C59" s="21">
         <f t="shared" ref="C59:F59" si="47">C47/$F47</f>
@@ -4884,7 +4894,7 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B60" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C60" s="21">
         <f t="shared" ref="C60:F60" si="49">C48/$F48</f>
@@ -4937,7 +4947,7 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B61" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C61" s="21">
         <f t="shared" ref="C61:F61" si="51">C49/$F49</f>
@@ -4990,7 +5000,7 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B62" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C62" s="21">
         <f t="shared" ref="C62:F62" si="53">C50/$F50</f>
@@ -5043,7 +5053,7 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B63" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C63" s="23">
         <f t="shared" ref="C63:F63" si="55">C51/$F51</f>
@@ -5096,7 +5106,7 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B64" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C64" s="17">
         <f t="shared" ref="C64:F64" si="57">C52/$F52</f>
@@ -5149,7 +5159,7 @@
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B66" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C66" s="32">
         <v>0</v>
@@ -5157,58 +5167,58 @@
     </row>
     <row r="68" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B68" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C68" s="29"/>
       <c r="D68" s="29"/>
       <c r="E68" s="29"/>
       <c r="F68" s="28"/>
       <c r="H68" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M68" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="M68" s="6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="69" spans="2:15" ht="15" x14ac:dyDescent="0.25">
       <c r="B69" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="C69" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C69" s="44" t="s">
+      <c r="D69" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D69" s="44" t="s">
+      <c r="E69" s="44" t="s">
         <v>18</v>
-      </c>
-      <c r="E69" s="44" t="s">
-        <v>19</v>
       </c>
       <c r="F69" s="45"/>
       <c r="G69" s="7"/>
       <c r="H69" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="I69" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="I69" s="44" t="s">
+      <c r="J69" s="44" t="s">
         <v>18</v>
-      </c>
-      <c r="J69" s="44" t="s">
-        <v>19</v>
       </c>
       <c r="K69" s="7"/>
       <c r="L69" s="7"/>
       <c r="M69" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="N69" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="N69" s="44" t="s">
+      <c r="O69" s="44" t="s">
         <v>18</v>
-      </c>
-      <c r="O69" s="44" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="70" spans="2:15" ht="15" x14ac:dyDescent="0.25">
       <c r="B70" s="30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C70" s="33">
         <f>[1]OnePerson!G31</f>
@@ -5241,7 +5251,7 @@
     </row>
     <row r="71" spans="2:15" ht="15" x14ac:dyDescent="0.25">
       <c r="B71" s="30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C71" s="36">
         <f>[1]OnePerson!G32</f>
@@ -5274,7 +5284,7 @@
     </row>
     <row r="72" spans="2:15" ht="15" x14ac:dyDescent="0.25">
       <c r="B72" s="30" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C72" s="36">
         <f>[1]OnePerson!G33</f>
@@ -5307,7 +5317,7 @@
     </row>
     <row r="73" spans="2:15" ht="15" x14ac:dyDescent="0.25">
       <c r="B73" s="30" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C73" s="36">
         <f>[1]OnePerson!G34</f>
@@ -5337,7 +5347,7 @@
     </row>
     <row r="74" spans="2:15" ht="15" x14ac:dyDescent="0.25">
       <c r="B74" s="30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C74" s="36">
         <f>[1]OnePerson!G35</f>
@@ -5367,7 +5377,7 @@
     </row>
     <row r="75" spans="2:15" ht="15" x14ac:dyDescent="0.25">
       <c r="B75" s="30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C75" s="36">
         <f>[1]OnePerson!G36</f>
@@ -5400,7 +5410,7 @@
     </row>
     <row r="76" spans="2:15" ht="15" x14ac:dyDescent="0.25">
       <c r="B76" s="30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C76" s="36">
         <f>[1]OnePerson!G37</f>
@@ -5433,7 +5443,7 @@
     </row>
     <row r="77" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B77" s="30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C77" s="38">
         <f>[1]OnePerson!G38</f>
@@ -5506,21 +5516,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -5645,7 +5655,7 @@
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="B1:M27"/>
+  <dimension ref="B1:M77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
@@ -5660,67 +5670,58 @@
   <sheetData>
     <row r="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="1"/>
+      <c r="B2" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="C2" s="1" t="s">
         <v>41</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>0</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="E2" s="1"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>597701.053643013</v>
+      <c r="C3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>461692.8424469239</v>
       </c>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E4">
-        <v>1510516.0951091901</v>
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1333929.1476687805</v>
       </c>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>987872.43858285202</v>
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>804895.68837679608</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -5728,48 +5729,42 @@
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>99715.360546481839</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M6" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>125376.86656725001</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7">
         <v>2</v>
       </c>
-      <c r="D7" t="s">
-        <v>2</v>
-      </c>
-      <c r="E7">
-        <v>302553.71482258302</v>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>287737.98222085688</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I7" s="4">
         <v>1</v>
@@ -5789,19 +5784,16 @@
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8">
-        <v>6</v>
-      </c>
-      <c r="C8">
         <v>2</v>
       </c>
-      <c r="D8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E8">
-        <v>225715.8401615</v>
+      <c r="C8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>208213.78607113534</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I8" s="4">
         <v>2</v>
@@ -5821,19 +5813,16 @@
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9">
-        <v>7</v>
-      </c>
-      <c r="C9">
         <v>3</v>
       </c>
-      <c r="D9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>78609.071429666597</v>
+      <c r="C9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>38223.680341122286</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I9" s="4">
         <v>3</v>
@@ -5853,19 +5842,16 @@
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10">
-        <v>8</v>
-      </c>
-      <c r="C10">
         <v>3</v>
       </c>
-      <c r="D10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E10">
-        <v>74331.568374583294</v>
+      <c r="C10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>97970.712003252251</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I10" s="4">
         <v>4</v>
@@ -5883,19 +5869,16 @@
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11">
-        <v>9</v>
-      </c>
-      <c r="C11">
         <v>3</v>
       </c>
-      <c r="D11" t="s">
-        <v>3</v>
-      </c>
-      <c r="E11">
-        <v>214926.651888416</v>
+      <c r="C11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>162794.76454298742</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I11" s="4">
         <v>5</v>
@@ -5913,19 +5896,16 @@
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12">
-        <v>10</v>
-      </c>
-      <c r="C12">
         <v>4</v>
       </c>
-      <c r="D12" t="s">
-        <v>1</v>
-      </c>
-      <c r="E12">
-        <v>242912.88811763801</v>
+      <c r="C12" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>175548.1377755001</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I12" s="4">
         <v>6</v>
@@ -5945,19 +5925,16 @@
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13">
-        <v>11</v>
-      </c>
-      <c r="C13">
         <v>4</v>
       </c>
-      <c r="D13" t="s">
-        <v>3</v>
-      </c>
-      <c r="E13">
-        <v>481043.68047886097</v>
+      <c r="C13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>429861.17069272167</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I13" s="4">
         <v>7</v>
@@ -5977,19 +5954,16 @@
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14">
-        <v>12</v>
-      </c>
-      <c r="C14">
         <v>5</v>
       </c>
-      <c r="D14" t="s">
-        <v>1</v>
-      </c>
-      <c r="E14">
-        <v>316730.200043466</v>
+      <c r="C14" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>302416.20874454407</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I14" s="4">
         <v>8</v>
@@ -6009,19 +5983,16 @@
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B15">
-        <v>13</v>
-      </c>
-      <c r="C15">
         <v>5</v>
       </c>
-      <c r="D15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E15">
-        <v>595161.53103013302</v>
+      <c r="C15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15">
+        <v>569846.47468317475</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J15" s="5">
         <v>1586052.5121910335</v>
@@ -6038,160 +6009,785 @@
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16">
-        <v>14</v>
-      </c>
-      <c r="C16">
         <v>6</v>
       </c>
-      <c r="D16" t="s">
-        <v>1</v>
-      </c>
-      <c r="E16" s="2">
+      <c r="C16" t="s">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2">
         <v>17630.20679</v>
       </c>
-      <c r="F16">
-        <v>119360.9876825</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" s="2">
+        <v>123094.58867</v>
+      </c>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="2">
+        <v>17712.811699999998</v>
+      </c>
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2">
+        <v>85466.730259999997</v>
+      </c>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1</v>
+      </c>
+      <c r="D20" s="2">
+        <v>665066.56470999995</v>
+      </c>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <v>7</v>
+      </c>
+      <c r="C21" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="2">
+        <v>64858.529419999999</v>
+      </c>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>8</v>
+      </c>
+      <c r="C22" t="s">
+        <v>0</v>
+      </c>
+      <c r="D22" s="2">
+        <v>121625.49533999999</v>
+      </c>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2">
+        <v>138048.92214000001</v>
+      </c>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <v>8</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2</v>
+      </c>
+      <c r="D24" s="2">
+        <v>145623.69245999999</v>
+      </c>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="70" t="s">
+        <v>42</v>
+      </c>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <v>20972.980538993601</v>
+      </c>
+      <c r="E30">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <v>101791.443381039</v>
+      </c>
+      <c r="E31">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32">
+        <v>56525.7782478925</v>
+      </c>
+      <c r="E32">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>9363.2104923139996</v>
+      </c>
+      <c r="E33">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>29187.200693063402</v>
+      </c>
+      <c r="E34">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>2</v>
+      </c>
+      <c r="D35">
+        <v>28107.324162689001</v>
+      </c>
+      <c r="E35">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>3</v>
+      </c>
+      <c r="C36" t="s">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>2587.17097574738</v>
+      </c>
+      <c r="E36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B37">
+        <v>3</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37">
+        <v>5272.2016418558496</v>
+      </c>
+      <c r="E37">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B38">
+        <v>3</v>
+      </c>
+      <c r="C38" t="s">
+        <v>2</v>
+      </c>
+      <c r="D38">
+        <v>14187.895576548101</v>
+      </c>
+      <c r="E38">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B39">
+        <v>4</v>
+      </c>
+      <c r="C39" t="s">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>10909.387874141699</v>
+      </c>
+      <c r="E39">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B40">
+        <v>4</v>
+      </c>
+      <c r="C40" t="s">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>38765.573310295011</v>
+      </c>
+      <c r="E40">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B41">
+        <v>5</v>
+      </c>
+      <c r="C41" t="s">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>34940.3033849606</v>
+      </c>
+      <c r="E41">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B42">
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>52565.235958389538</v>
+      </c>
+      <c r="E42">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B43">
+        <v>6</v>
+      </c>
+      <c r="C43" t="s">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>3795.8709036518198</v>
+      </c>
+      <c r="E43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B44">
+        <v>6</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1</v>
+      </c>
+      <c r="D44">
+        <v>6531.0686161737603</v>
+      </c>
+      <c r="E44">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B45">
+        <v>6</v>
+      </c>
+      <c r="C45" t="s">
+        <v>2</v>
+      </c>
+      <c r="D45">
+        <v>4233.5977867305201</v>
+      </c>
+      <c r="E45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B46">
+        <v>7</v>
+      </c>
+      <c r="C46" t="s">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>31643.1944620621</v>
+      </c>
+      <c r="E46">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B47">
+        <v>7</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1</v>
+      </c>
+      <c r="D47">
+        <v>14117.8259404212</v>
+      </c>
+      <c r="E47">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B48">
+        <v>7</v>
+      </c>
+      <c r="C48" t="s">
+        <v>2</v>
+      </c>
+      <c r="D48">
+        <v>16081.6986499751</v>
+      </c>
+      <c r="E48">
         <v>15</v>
       </c>
-      <c r="C17">
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B49">
+        <v>8</v>
+      </c>
+      <c r="C49" t="s">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>20577.984808375099</v>
+      </c>
+      <c r="E49">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B50">
+        <v>8</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1</v>
+      </c>
+      <c r="D50">
+        <v>8248.9312060110606</v>
+      </c>
+      <c r="E50">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B51">
+        <v>8</v>
+      </c>
+      <c r="C51" t="s">
+        <v>2</v>
+      </c>
+      <c r="D51">
+        <v>4558.7508507235698</v>
+      </c>
+      <c r="E51">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B53" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B54" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>40</v>
+      </c>
+      <c r="C55" t="s">
+        <v>41</v>
+      </c>
+      <c r="D55" t="s">
+        <v>43</v>
+      </c>
+      <c r="E55" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>0</v>
+      </c>
+      <c r="D56">
+        <v>63549.153434615902</v>
+      </c>
+      <c r="E56">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1</v>
+      </c>
+      <c r="D57">
+        <v>210535.026176057</v>
+      </c>
+      <c r="E57">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>2</v>
+      </c>
+      <c r="D58">
+        <v>121351.542268502</v>
+      </c>
+      <c r="E58">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B59">
+        <v>2</v>
+      </c>
+      <c r="C59" t="s">
+        <v>0</v>
+      </c>
+      <c r="D59">
+        <v>20968.7890230091</v>
+      </c>
+      <c r="E59">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B60">
+        <v>2</v>
+      </c>
+      <c r="C60" t="s">
+        <v>1</v>
+      </c>
+      <c r="D60">
+        <v>62137.604970189903</v>
+      </c>
+      <c r="E60">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B61">
+        <v>2</v>
+      </c>
+      <c r="C61" t="s">
+        <v>2</v>
+      </c>
+      <c r="D61">
+        <v>56617.428037848404</v>
+      </c>
+      <c r="E61">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>0</v>
+      </c>
+      <c r="D62">
+        <v>4916.5079167325503</v>
+      </c>
+      <c r="E62">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="63" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1</v>
+      </c>
+      <c r="D63">
+        <v>11219.7352089292</v>
+      </c>
+      <c r="E63">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>2</v>
+      </c>
+      <c r="D64">
+        <v>30372.661147028601</v>
+      </c>
+      <c r="E64">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B65">
+        <v>4</v>
+      </c>
+      <c r="C65" t="s">
+        <v>0</v>
+      </c>
+      <c r="D65">
+        <v>33377.814186217001</v>
+      </c>
+      <c r="E65">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B66">
+        <v>4</v>
+      </c>
+      <c r="C66" t="s">
+        <v>2</v>
+      </c>
+      <c r="D66">
+        <v>70367.585458441914</v>
+      </c>
+      <c r="E66">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B67">
+        <v>5</v>
+      </c>
+      <c r="C67" t="s">
+        <v>0</v>
+      </c>
+      <c r="D67">
+        <v>69883.099397594095</v>
+      </c>
+      <c r="E67">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B68">
+        <v>5</v>
+      </c>
+      <c r="C68" t="s">
+        <v>2</v>
+      </c>
+      <c r="D68">
+        <v>132239.30044086539</v>
+      </c>
+      <c r="E68">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="69" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B69">
         <v>6</v>
       </c>
-      <c r="D17" t="s">
+      <c r="C69" t="s">
+        <v>0</v>
+      </c>
+      <c r="D69">
+        <v>7719.92068896827</v>
+      </c>
+      <c r="E69">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B70">
+        <v>6</v>
+      </c>
+      <c r="C70" t="s">
+        <v>1</v>
+      </c>
+      <c r="D70">
+        <v>6670.6837531622796</v>
+      </c>
+      <c r="E70">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="71" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B71">
+        <v>6</v>
+      </c>
+      <c r="C71" t="s">
         <v>2</v>
       </c>
-      <c r="E17" s="2">
-        <v>123094.58867</v>
-      </c>
-      <c r="F17">
-        <v>39331.568567000002</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18">
-        <v>16</v>
-      </c>
-      <c r="C18">
-        <v>6</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="D71">
+        <v>4233.5977867305201</v>
+      </c>
+      <c r="E71">
         <v>3</v>
       </c>
-      <c r="E18" s="2">
-        <v>17712.811699999998</v>
-      </c>
-      <c r="F18">
-        <v>41087.375039166604</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19">
-        <v>17</v>
-      </c>
-      <c r="C19">
+    </row>
+    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B72">
         <v>7</v>
       </c>
-      <c r="D19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E19" s="2">
-        <v>85466.730259999997</v>
-      </c>
-      <c r="F19">
-        <v>569393.78630000004</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20">
-        <v>18</v>
-      </c>
-      <c r="C20">
+      <c r="C72" t="s">
+        <v>0</v>
+      </c>
+      <c r="D72">
+        <v>47157.520468889401</v>
+      </c>
+      <c r="E72">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="73" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B73">
         <v>7</v>
       </c>
-      <c r="D20" t="s">
+      <c r="C73" t="s">
+        <v>1</v>
+      </c>
+      <c r="D73">
+        <v>27508.592579624699</v>
+      </c>
+      <c r="E73">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="74" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B74">
+        <v>7</v>
+      </c>
+      <c r="C74" t="s">
         <v>2</v>
       </c>
-      <c r="E20" s="2">
-        <v>665066.56470999995</v>
-      </c>
-      <c r="F20">
-        <v>97527.679770000002</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21">
-        <v>19</v>
-      </c>
-      <c r="C21">
+      <c r="D74">
+        <v>26449.980666032399</v>
+      </c>
+      <c r="E74">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B75">
+        <v>8</v>
+      </c>
+      <c r="C75" t="s">
+        <v>0</v>
+      </c>
+      <c r="D75">
+        <v>31749.7412333293</v>
+      </c>
+      <c r="E75">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="76" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B76">
+        <v>8</v>
+      </c>
+      <c r="C76" t="s">
+        <v>1</v>
+      </c>
+      <c r="D76">
+        <v>13066.8121666193</v>
+      </c>
+      <c r="E76">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B77">
+        <v>8</v>
+      </c>
+      <c r="C77" t="s">
+        <v>2</v>
+      </c>
+      <c r="D77">
+        <v>11381.3647679572</v>
+      </c>
+      <c r="E77">
         <v>7</v>
-      </c>
-      <c r="D21" t="s">
-        <v>3</v>
-      </c>
-      <c r="E21" s="2">
-        <v>64858.529419999999</v>
-      </c>
-      <c r="F21">
-        <v>259749.11470000001</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22">
-        <v>20</v>
-      </c>
-      <c r="C22">
-        <v>8</v>
-      </c>
-      <c r="D22" t="s">
-        <v>1</v>
-      </c>
-      <c r="E22" s="2">
-        <v>121625.49533999999</v>
-      </c>
-      <c r="F22">
-        <v>296446.54610749998</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23">
-        <v>21</v>
-      </c>
-      <c r="C23">
-        <v>8</v>
-      </c>
-      <c r="D23" t="s">
-        <v>2</v>
-      </c>
-      <c r="E23" s="2">
-        <v>138048.92214000001</v>
-      </c>
-      <c r="F23">
-        <v>24109.207162333299</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24">
-        <v>22</v>
-      </c>
-      <c r="C24">
-        <v>8</v>
-      </c>
-      <c r="D24" t="s">
-        <v>3</v>
-      </c>
-      <c r="E24" s="2">
-        <v>145623.69245999999</v>
-      </c>
-      <c r="F24">
-        <v>44467.608008833296</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="70" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -6217,12 +6813,12 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="67" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="73" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B2" s="73"/>
       <c r="C2" s="73"/>
@@ -6237,19 +6833,19 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="50" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="59" t="s">
+      <c r="C3" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="59" t="s">
+      <c r="D3" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="E3" s="59" t="s">
         <v>19</v>
-      </c>
-      <c r="E3" s="59" t="s">
-        <v>20</v>
       </c>
       <c r="F3" s="59"/>
       <c r="I3" s="54"/>
@@ -6259,7 +6855,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="50" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="62">
         <v>2245780.8484</v>
@@ -6285,7 +6881,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="50" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="62">
         <v>198527.93961</v>
@@ -6311,7 +6907,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="50" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="62">
         <v>204361.06034</v>
@@ -6337,7 +6933,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="50" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="62">
         <v>0</v>
@@ -6364,7 +6960,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="50" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="62">
         <v>0</v>
@@ -6391,7 +6987,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="50" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" s="62">
         <v>132569.66722999999</v>
@@ -6417,7 +7013,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="62">
         <v>782213.25051000004</v>
@@ -6443,7 +7039,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="50" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="62">
         <v>201049.04508000001</v>
@@ -6469,7 +7065,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="50" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" s="62">
         <v>3880764.3125</v>
@@ -6503,7 +7099,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="73" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" s="73"/>
       <c r="C14" s="73"/>
@@ -6518,19 +7114,19 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="50" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="59" t="s">
+      <c r="C15" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="59" t="s">
+      <c r="D15" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="59" t="s">
+      <c r="E15" s="59" t="s">
         <v>19</v>
-      </c>
-      <c r="E15" s="59" t="s">
-        <v>20</v>
       </c>
       <c r="F15" s="59"/>
       <c r="I15" s="54"/>
@@ -6540,7 +7136,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="50" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B16" s="58">
         <f t="shared" ref="B16:E24" si="1">B4/$E4</f>
@@ -6566,7 +7162,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="50" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B17" s="58">
         <f t="shared" si="1"/>
@@ -6592,7 +7188,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="50" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B18" s="58">
         <f t="shared" si="1"/>
@@ -6618,7 +7214,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="50" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B19" s="58">
         <f t="shared" si="1"/>
@@ -6644,7 +7240,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="50" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B20" s="58">
         <f t="shared" si="1"/>
@@ -6670,7 +7266,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="50" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21" s="58">
         <f t="shared" si="1"/>
@@ -6696,7 +7292,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B22" s="58">
         <f t="shared" si="1"/>
@@ -6722,7 +7318,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="50" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B23" s="58">
         <f t="shared" si="1"/>
@@ -6748,7 +7344,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="50" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B24" s="58">
         <f t="shared" si="1"/>
@@ -6777,7 +7373,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="71" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B27" s="71"/>
       <c r="C27" s="71"/>
@@ -6792,22 +7388,22 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="54" t="s">
+      <c r="C28" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="54" t="s">
+      <c r="D28" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="D28" s="54" t="s">
+      <c r="E28" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="E28" s="54" t="s">
-        <v>20</v>
-      </c>
       <c r="F28" s="54" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I28" s="54"/>
       <c r="J28" s="54"/>
@@ -6816,7 +7412,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="46" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B29" s="72">
         <v>0.79</v>
@@ -6841,7 +7437,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="46" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B30" s="72"/>
       <c r="C30" s="72"/>
@@ -6855,7 +7451,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="46" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B31" s="55">
         <v>0.7</v>
@@ -6880,7 +7476,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="46" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B32" s="72">
         <v>0</v>
@@ -6905,7 +7501,7 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="46" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B33" s="72"/>
       <c r="C33" s="72"/>
@@ -6919,7 +7515,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="46" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B34" s="72">
         <v>0.65</v>
@@ -6944,7 +7540,7 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="46" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B35" s="72"/>
       <c r="C35" s="72"/>
@@ -6958,7 +7554,7 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="46" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B36" s="72"/>
       <c r="C36" s="72"/>
@@ -6972,7 +7568,7 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="46" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B37" s="55">
         <f>SUMPRODUCT(B29:B36,$F29:$F36)</f>
@@ -7007,22 +7603,22 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="B40" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="54" t="s">
+      <c r="C40" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="C40" s="54" t="s">
+      <c r="D40" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="D40" s="54" t="s">
+      <c r="E40" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="E40" s="54" t="s">
-        <v>20</v>
-      </c>
       <c r="F40" s="54" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H40" s="71"/>
       <c r="I40" s="71"/>
@@ -7032,7 +7628,7 @@
     </row>
     <row r="41" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="46" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B41" s="53">
         <f t="shared" ref="B41:D42" si="2">B4*B$29/(SUM(B$4:B$5)/SUM($E$4:$E$5))*$F$29/($F$4+$F$5)</f>
@@ -7059,7 +7655,7 @@
     </row>
     <row r="42" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A42" s="46" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B42" s="53">
         <f t="shared" si="2"/>
@@ -7088,7 +7684,7 @@
     </row>
     <row r="43" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A43" s="46" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B43" s="53">
         <f>B6*B31/B18*$F$31/$F$6</f>
@@ -7117,7 +7713,7 @@
     </row>
     <row r="44" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A44" s="46" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B44" s="53">
         <v>0</v>
@@ -7145,7 +7741,7 @@
     </row>
     <row r="45" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A45" s="46" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B45" s="53">
         <v>0</v>
@@ -7173,7 +7769,7 @@
     </row>
     <row r="46" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A46" s="46" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B46" s="53">
         <f t="shared" ref="B46:D48" si="5">B9*B$34/(SUM(B$9:B$11)/SUM($E$9:$E$11))*$F$34/($F$9+$F$10+$F$11)</f>
@@ -7202,7 +7798,7 @@
     </row>
     <row r="47" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A47" s="46" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B47" s="53">
         <f t="shared" si="5"/>
@@ -7231,7 +7827,7 @@
     </row>
     <row r="48" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A48" s="46" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B48" s="53">
         <f t="shared" si="5"/>
@@ -7260,7 +7856,7 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="46" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B49" s="53">
         <f>SUM(B41:B48)</f>
@@ -7546,7 +8142,7 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" s="48" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B63" s="48"/>
       <c r="C63" s="48"/>
@@ -7556,7 +8152,7 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="48" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B64" s="47">
         <f>SUM(B41:B42)/SUM($E$41:$E$42)</f>
@@ -7586,7 +8182,7 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="48" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B65" s="47">
         <f>B43/$E$43</f>
@@ -7611,7 +8207,7 @@
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" s="48" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B66" s="47">
         <f>SUM(B44:B45)/SUM($E$44:$E$45)</f>
@@ -7639,7 +8235,7 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" s="48" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B67" s="47">
         <f>SUM(B46:B48)/SUM($E$46:$E$48)</f>
@@ -7667,7 +8263,7 @@
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" s="48" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B68" s="47">
         <f>B49/$E$49</f>

</xml_diff>

<commit_message>
Updated calibration targets to aligned with travel-diary-survey-tools (commit id:  61f48bf0c682899b4ae2815c585ea50cfbcd4194)
Adjusted calibration targets to account for:
- Changes to tour purpose hierarchy
- Added ferry as one of the transit mode choice for calibration
</commit_message>
<xml_diff>
--- a/utilities/calibration/workbook_templates/04_CoordinatedDailyActivityPattern_2023_blank.xlsx
+++ b/utilities/calibration/workbook_templates/04_CoordinatedDailyActivityPattern_2023_blank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\travel-model-one\utilities\calibration\workbook_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C1F13A-4898-48DB-90CD-1A7ABDD79E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{224AA7D1-6253-4440-8332-3EA899DB7DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="49">
   <si>
     <t>H</t>
   </si>
@@ -239,13 +239,7 @@
     <t>activity_pattern</t>
   </si>
   <si>
-    <t xml:space="preserve">**BATS 2023 was under-reporting mandatory tours for students under 18, most likely due to proxy reporting. As a result, we will not be using BATS CDAP share for students under 18 and keep the targets from the previous calibration </t>
-  </si>
-  <si>
     <t>num_pers</t>
-  </si>
-  <si>
-    <t>Source: M:/Development/Travel Model One/Calibration/Version 1.7/2023_BATS_Summaries/pipeline_mt_20260623_NoMon_rmo/ctramp_2023/BATS_Summaries/dap_summaries.csv</t>
   </si>
   <si>
     <t>num_records</t>
@@ -261,6 +255,9 @@
   </si>
   <si>
     <t>Source: M:/Development/Travel Model One/Calibration/Version 1.7/2023_BATS_Summaries/pipeline_mt_20260623_NoMon_rmo/ctramp_2023/BATS_Summaries/BATS2023_person_type_summary_north_bay.csv</t>
+  </si>
+  <si>
+    <t>Source: M:/Development/Travel Model One/Calibration/Version 1.7/2023_BATS_Summaries/pipeline_mt_20260821_NoMon_rmo/ctramp_2023/BATS_Summaries/dap_summaries.csv</t>
   </si>
 </sst>
 </file>
@@ -600,13 +597,13 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -5670,7 +5667,7 @@
   <sheetData>
     <row r="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
@@ -5681,7 +5678,7 @@
         <v>41</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E2" s="1"/>
     </row>
@@ -5693,7 +5690,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>461692.8424469239</v>
+        <v>461223.06254459248</v>
       </c>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
@@ -5704,7 +5701,7 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <v>1333929.1476687805</v>
+        <v>1319053.0998245263</v>
       </c>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
@@ -5715,7 +5712,7 @@
         <v>2</v>
       </c>
       <c r="D5">
-        <v>804895.68837679608</v>
+        <v>820108.86244772957</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>6</v>
@@ -5735,7 +5732,7 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <v>99715.360546481839</v>
+        <v>100056.63644374204</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>3</v>
@@ -5761,7 +5758,7 @@
         <v>1</v>
       </c>
       <c r="D7">
-        <v>287737.98222085688</v>
+        <v>275488.69364808826</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>7</v>
@@ -5790,7 +5787,7 @@
         <v>2</v>
       </c>
       <c r="D8">
-        <v>208213.78607113534</v>
+        <v>220121.79874664376</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>8</v>
@@ -5819,7 +5816,7 @@
         <v>0</v>
       </c>
       <c r="D9">
-        <v>38223.680341122286</v>
+        <v>38280.722291383849</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>9</v>
@@ -5848,7 +5845,7 @@
         <v>1</v>
       </c>
       <c r="D10">
-        <v>97970.712003252251</v>
+        <v>94740.132726467826</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>10</v>
@@ -5875,7 +5872,7 @@
         <v>2</v>
       </c>
       <c r="D11">
-        <v>162794.76454298742</v>
+        <v>165968.30186951029</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>11</v>
@@ -5902,7 +5899,7 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <v>175548.1377755001</v>
+        <v>186265.85543595851</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>12</v>
@@ -5928,10 +5925,10 @@
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13">
-        <v>429861.17069272167</v>
+        <v>1595.3973574861745</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>13</v>
@@ -5954,13 +5951,13 @@
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D14">
-        <v>302416.20874454407</v>
+        <v>417548.05567477713</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>14</v>
@@ -5986,10 +5983,10 @@
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D15">
-        <v>569846.47468317475</v>
+        <v>304188.31656060548</v>
       </c>
       <c r="I15" s="4" t="s">
         <v>4</v>
@@ -6009,24 +6006,24 @@
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="2">
-        <v>17630.20679</v>
+        <v>5095.9923076611367</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="2">
-        <v>123094.58867</v>
+        <v>562978.37455945229</v>
       </c>
       <c r="E17" s="2"/>
     </row>
@@ -6035,34 +6032,34 @@
         <v>6</v>
       </c>
       <c r="C18" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D18" s="2">
-        <v>17712.811699999998</v>
+        <v>41115.091661171064</v>
       </c>
       <c r="E18" s="2"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" s="2">
-        <v>85466.730259999997</v>
+        <v>32780.663158173164</v>
       </c>
       <c r="E19" s="2"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="2">
-        <v>665066.56470999995</v>
+        <v>41918.179611378931</v>
       </c>
       <c r="E20" s="2"/>
     </row>
@@ -6071,34 +6068,34 @@
         <v>7</v>
       </c>
       <c r="C21" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2">
-        <v>64858.529419999999</v>
+        <v>247900.7678317161</v>
       </c>
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="2">
-        <v>121625.49533999999</v>
+        <v>140853.46659383521</v>
       </c>
       <c r="E22" s="2"/>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="2">
-        <v>138048.92214000001</v>
+        <v>140850.42326779067</v>
       </c>
       <c r="E23" s="2"/>
     </row>
@@ -6107,22 +6104,39 @@
         <v>8</v>
       </c>
       <c r="C24" t="s">
+        <v>0</v>
+      </c>
+      <c r="D24" s="2">
+        <v>157345.89475843927</v>
+      </c>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="70">
+        <v>8</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>64377.458058831013</v>
+      </c>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26">
+        <v>8</v>
+      </c>
+      <c r="C26" t="s">
         <v>2</v>
       </c>
-      <c r="D24" s="2">
-        <v>145623.69245999999</v>
-      </c>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B25" s="70" t="s">
-        <v>42</v>
-      </c>
-      <c r="E25" s="2"/>
+      <c r="D26">
+        <v>39919.065974013021</v>
+      </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -6130,7 +6144,7 @@
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -6144,10 +6158,10 @@
         <v>41</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.25">
@@ -6460,12 +6474,12 @@
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B54" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.25">
@@ -6476,10 +6490,10 @@
         <v>41</v>
       </c>
       <c r="D55" t="s">
+        <v>42</v>
+      </c>
+      <c r="E55" t="s">
         <v>43</v>
-      </c>
-      <c r="E55" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.25">
@@ -6817,19 +6831,19 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="72" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
       <c r="F2" s="60"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="50" t="s">
@@ -7098,19 +7112,19 @@
       <c r="F13" s="50"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="73" t="s">
+      <c r="A14" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="73"/>
-      <c r="C14" s="73"/>
-      <c r="D14" s="73"/>
-      <c r="E14" s="73"/>
+      <c r="B14" s="72"/>
+      <c r="C14" s="72"/>
+      <c r="D14" s="72"/>
+      <c r="E14" s="72"/>
       <c r="F14" s="60"/>
-      <c r="H14" s="71"/>
-      <c r="I14" s="71"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="71"/>
-      <c r="L14" s="71"/>
+      <c r="H14" s="73"/>
+      <c r="I14" s="73"/>
+      <c r="J14" s="73"/>
+      <c r="K14" s="73"/>
+      <c r="L14" s="73"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="50" t="s">
@@ -7372,19 +7386,19 @@
       <c r="A25" s="57"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="71" t="s">
+      <c r="A27" s="73" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="71"/>
-      <c r="C27" s="71"/>
-      <c r="D27" s="71"/>
-      <c r="E27" s="71"/>
+      <c r="B27" s="73"/>
+      <c r="C27" s="73"/>
+      <c r="D27" s="73"/>
+      <c r="E27" s="73"/>
       <c r="F27" s="56"/>
-      <c r="H27" s="71"/>
-      <c r="I27" s="71"/>
-      <c r="J27" s="71"/>
-      <c r="K27" s="71"/>
-      <c r="L27" s="71"/>
+      <c r="H27" s="73"/>
+      <c r="I27" s="73"/>
+      <c r="J27" s="73"/>
+      <c r="K27" s="73"/>
+      <c r="L27" s="73"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="46" t="s">
@@ -7414,20 +7428,20 @@
       <c r="A29" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B29" s="72">
+      <c r="B29" s="71">
         <v>0.79</v>
       </c>
-      <c r="C29" s="72">
+      <c r="C29" s="71">
         <v>0.12</v>
       </c>
-      <c r="D29" s="72">
+      <c r="D29" s="71">
         <v>0.09</v>
       </c>
-      <c r="E29" s="72">
+      <c r="E29" s="71">
         <f>SUM(B29:D29)</f>
         <v>1</v>
       </c>
-      <c r="F29" s="72">
+      <c r="F29" s="71">
         <v>0.47599999999999998</v>
       </c>
       <c r="I29" s="64"/>
@@ -7439,11 +7453,11 @@
       <c r="A30" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="72"/>
-      <c r="C30" s="72"/>
-      <c r="D30" s="72"/>
-      <c r="E30" s="72"/>
-      <c r="F30" s="72"/>
+      <c r="B30" s="71"/>
+      <c r="C30" s="71"/>
+      <c r="D30" s="71"/>
+      <c r="E30" s="71"/>
+      <c r="F30" s="71"/>
       <c r="I30" s="64"/>
       <c r="J30" s="64"/>
       <c r="K30" s="64"/>
@@ -7478,20 +7492,20 @@
       <c r="A32" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="72">
-        <v>0</v>
-      </c>
-      <c r="C32" s="72">
+      <c r="B32" s="71">
+        <v>0</v>
+      </c>
+      <c r="C32" s="71">
         <v>0.8</v>
       </c>
-      <c r="D32" s="72">
+      <c r="D32" s="71">
         <v>0.2</v>
       </c>
-      <c r="E32" s="72">
+      <c r="E32" s="71">
         <f>SUM(B32:D32)</f>
         <v>1</v>
       </c>
-      <c r="F32" s="72">
+      <c r="F32" s="71">
         <v>0.22600000000000001</v>
       </c>
       <c r="I32" s="64"/>
@@ -7503,11 +7517,11 @@
       <c r="A33" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="72"/>
-      <c r="C33" s="72"/>
-      <c r="D33" s="72"/>
-      <c r="E33" s="72"/>
-      <c r="F33" s="72"/>
+      <c r="B33" s="71"/>
+      <c r="C33" s="71"/>
+      <c r="D33" s="71"/>
+      <c r="E33" s="71"/>
+      <c r="F33" s="71"/>
       <c r="I33" s="64"/>
       <c r="J33" s="64"/>
       <c r="K33" s="64"/>
@@ -7517,20 +7531,20 @@
       <c r="A34" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="72">
+      <c r="B34" s="71">
         <v>0.65</v>
       </c>
-      <c r="C34" s="72">
+      <c r="C34" s="71">
         <v>0.2</v>
       </c>
-      <c r="D34" s="72">
+      <c r="D34" s="71">
         <v>0.15</v>
       </c>
-      <c r="E34" s="72">
+      <c r="E34" s="71">
         <f>SUM(B34:D34)</f>
         <v>1</v>
       </c>
-      <c r="F34" s="72">
+      <c r="F34" s="71">
         <v>0.246</v>
       </c>
       <c r="I34" s="64"/>
@@ -7542,11 +7556,11 @@
       <c r="A35" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="72"/>
-      <c r="C35" s="72"/>
-      <c r="D35" s="72"/>
-      <c r="E35" s="72"/>
-      <c r="F35" s="72"/>
+      <c r="B35" s="71"/>
+      <c r="C35" s="71"/>
+      <c r="D35" s="71"/>
+      <c r="E35" s="71"/>
+      <c r="F35" s="71"/>
       <c r="I35" s="64"/>
       <c r="J35" s="64"/>
       <c r="K35" s="64"/>
@@ -7556,11 +7570,11 @@
       <c r="A36" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="72"/>
-      <c r="C36" s="72"/>
-      <c r="D36" s="72"/>
-      <c r="E36" s="72"/>
-      <c r="F36" s="72"/>
+      <c r="B36" s="71"/>
+      <c r="C36" s="71"/>
+      <c r="D36" s="71"/>
+      <c r="E36" s="71"/>
+      <c r="F36" s="71"/>
       <c r="I36" s="64"/>
       <c r="J36" s="64"/>
       <c r="K36" s="64"/>
@@ -7620,11 +7634,11 @@
       <c r="F40" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="H40" s="71"/>
-      <c r="I40" s="71"/>
-      <c r="J40" s="71"/>
-      <c r="K40" s="71"/>
-      <c r="L40" s="71"/>
+      <c r="H40" s="73"/>
+      <c r="I40" s="73"/>
+      <c r="J40" s="73"/>
+      <c r="K40" s="73"/>
+      <c r="L40" s="73"/>
     </row>
     <row r="41" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="46" t="s">
@@ -7912,11 +7926,11 @@
         <f>E40</f>
         <v>Total</v>
       </c>
-      <c r="H52" s="71"/>
-      <c r="I52" s="71"/>
-      <c r="J52" s="71"/>
-      <c r="K52" s="71"/>
-      <c r="L52" s="71"/>
+      <c r="H52" s="73"/>
+      <c r="I52" s="73"/>
+      <c r="J52" s="73"/>
+      <c r="K52" s="73"/>
+      <c r="L52" s="73"/>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="50" t="str">
@@ -8174,11 +8188,11 @@
         <f>SUM(E41:E42)/$E$49</f>
         <v>0.47599999999999992</v>
       </c>
-      <c r="H64" s="71"/>
-      <c r="I64" s="71"/>
-      <c r="J64" s="71"/>
-      <c r="K64" s="71"/>
-      <c r="L64" s="71"/>
+      <c r="H64" s="73"/>
+      <c r="I64" s="73"/>
+      <c r="J64" s="73"/>
+      <c r="K64" s="73"/>
+      <c r="L64" s="73"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="48" t="s">
@@ -8316,17 +8330,12 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="H14:L14"/>
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="H52:L52"/>
+    <mergeCell ref="H64:L64"/>
+    <mergeCell ref="H40:L40"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="F34:F36"/>
     <mergeCell ref="E32:E33"/>
     <mergeCell ref="H27:L27"/>
     <mergeCell ref="F29:F30"/>
@@ -8334,12 +8343,17 @@
     <mergeCell ref="D29:D30"/>
     <mergeCell ref="D32:D33"/>
     <mergeCell ref="E29:E30"/>
-    <mergeCell ref="H52:L52"/>
-    <mergeCell ref="H64:L64"/>
-    <mergeCell ref="H40:L40"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="F34:F36"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="H14:L14"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="C34:C36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>